<commit_message>
Update quotation system and onboarding
</commit_message>
<xml_diff>
--- a/data/quotation_items.xlsx
+++ b/data/quotation_items.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AE2"/>
+  <dimension ref="A1:AE3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -589,9 +589,104 @@
         <v>2026-05-31T15:32:14.427Z</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>960d0a17-a802-4dc1-aa7f-74f05fb117da</v>
+      </c>
+      <c r="B3" t="str">
+        <v>5877fe16-3734-4276-bfee-1a380882f18d</v>
+      </c>
+      <c r="C3" t="str">
+        <v>DEMO-001</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Demo Motor</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>700</v>
+      </c>
+      <c r="G3">
+        <v>700</v>
+      </c>
+      <c r="H3">
+        <v>619.469</v>
+      </c>
+      <c r="I3">
+        <v>80.531</v>
+      </c>
+      <c r="J3" t="str">
+        <v>sea</v>
+      </c>
+      <c r="K3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L3">
+        <v>160</v>
+      </c>
+      <c r="M3">
+        <v>779.469</v>
+      </c>
+      <c r="N3">
+        <v>109.7844</v>
+      </c>
+      <c r="O3">
+        <v>10</v>
+      </c>
+      <c r="P3">
+        <v>10.9784</v>
+      </c>
+      <c r="Q3">
+        <v>3.2935</v>
+      </c>
+      <c r="R3">
+        <v>1.0978</v>
+      </c>
+      <c r="S3">
+        <v>100</v>
+      </c>
+      <c r="T3">
+        <v>0</v>
+      </c>
+      <c r="U3">
+        <v>225.1542</v>
+      </c>
+      <c r="V3">
+        <v>225.1542</v>
+      </c>
+      <c r="W3">
+        <v>247.6696</v>
+      </c>
+      <c r="X3">
+        <v>22.5154</v>
+      </c>
+      <c r="Y3">
+        <v>9.0909</v>
+      </c>
+      <c r="Z3">
+        <v>4.9534</v>
+      </c>
+      <c r="AA3">
+        <v>10</v>
+      </c>
+      <c r="AB3" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC3" t="str">
+        <v>ee86473c-b3ba-44fc-9656-9f4bd7e43d1d</v>
+      </c>
+      <c r="AD3" t="str">
+        <v>2026-05-31T17:01:07.386Z</v>
+      </c>
+      <c r="AE3" t="str">
+        <v>2026-05-31T17:01:07.386Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AE2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AE3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>